<commit_message>
chore(asistentes): actualizar plantilla Excel de importacion
</commit_message>
<xml_diff>
--- a/assets/plantilla-asistentes.xlsx
+++ b/assets/plantilla-asistentes.xlsx
@@ -8,7 +8,8 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\1. Aplicaciones\BAUTISMOS\Grupos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CDCE10B-BBD4-43AB-A62F-0FFB69A57236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{808B2BAC-6C29-45AE-9787-B65F86217745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="iwPxcn3KqJiXtoRv8hXpE7OsvL4xmcY1y6zXzHuT+cbHPl5lxGVNKotyQDUq2NGLkn2cqnSpRiUBJLrIzSfAOg==" workbookSaltValue="kXJ5w/Ur2+gCHmJ7Jxy7yg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10446,7 +10447,7 @@
       <c r="C1800" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="9ytc4GpnwuzkAzi9l+w2OF8o4vJl7S1vA8eJ/TyH98t1wKknTYsUpJ0grY4rU9a/Yf1anm5GxStJBxz0Qyj+3g==" saltValue="XtA3y0iMcVFiUOpw5t+BMA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="7BEDt7SSjWka/vdv3sgdDSP5YyKqeExHvLCD0qSlOz3M7n2YlCl5XXs8Hf1lbxmGy30IU2hmp8X0YCIIvg/awg==" saltValue="awKPfMAj1U6447vzeKAocw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <dataValidations count="3">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="B2:B1000" xr:uid="{5A402809-390D-4D0C-B229-80A8C4978C07}">
       <formula1>"Alumno,Responsable de grupo,General"</formula1>
@@ -10455,7 +10456,7 @@
       <formula1>"de 3 a 5 años,de 6 a 9 años,de 10 a 14 años, de 15 a 18 años, mayor de 18 años"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1000" xr:uid="{D73920EE-18B4-4753-BE7B-11E17A8CA3B4}">
-      <formula1>"Prescolar,Infantil,Primaria,Secundaria,Bachiller/FP,Estudios Superiores"</formula1>
+      <formula1>"No corresponde,Preescolar,Infantil,Primaria,Secundaria,Bachiller/FP,Estudios Superiores"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>